<commit_message>
identificação para saldo baixo em estoque.
Ao estoque ficar com saldo abaixo de 20%, a linha do produto com esse status ficará com uma coloração diferenciada, assim facilitando a identificação para ação de procedimento de compra.
</commit_message>
<xml_diff>
--- a/planilha de controle de estoque.xlsx
+++ b/planilha de controle de estoque.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Odirlei Guilherme\Desktop\controle_de_estoque_basico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C57ED36-687F-4B74-95E0-01E5F134A0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{11A3E976-6574-4C9F-9A17-EC0406ED2E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20280" yWindow="-135" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{FB90DC12-CE7E-421E-A7F9-F06FD8601840}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="25">
   <si>
     <t>Produto</t>
   </si>
@@ -200,7 +200,20 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -228,12 +241,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{36F923C0-43EC-4309-9C6B-28398D46868F}" name="Tabela5" displayName="Tabela5" ref="B2:E24" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="B2:E24" xr:uid="{36F923C0-43EC-4309-9C6B-28398D46868F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{36F923C0-43EC-4309-9C6B-28398D46868F}" name="Tabela5" displayName="Tabela5" ref="B2:E27" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="B2:E27" xr:uid="{36F923C0-43EC-4309-9C6B-28398D46868F}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{9A824ECF-4997-4FB3-8467-CA5F746211D1}" name="Data" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{6F519A01-4485-4303-A5F9-1109AE4DC2DA}" name="Produto" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{F0E480FA-F451-40F8-AC3B-1DC003CAD38F}" name="Status " dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{9A824ECF-4997-4FB3-8467-CA5F746211D1}" name="Data" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{6F519A01-4485-4303-A5F9-1109AE4DC2DA}" name="Produto" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{F0E480FA-F451-40F8-AC3B-1DC003CAD38F}" name="Status " dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{853DA4E0-565B-4E84-ACE2-FAB8B85CA4C3}" name="Quantidade"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -537,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{137AD64A-E144-47FE-A0E9-95F7C892ACF1}">
-  <dimension ref="B2:F24"/>
+  <dimension ref="B2:F27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -858,7 +871,7 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="4">
-        <v>46023</v>
+        <v>46327</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>18</v>
@@ -869,6 +882,39 @@
       <c r="E24" s="2">
         <v>12</v>
       </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="4">
+        <v>46327</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" s="2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="4">
+        <v>46327</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="4"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1030,15 +1076,15 @@
       </c>
       <c r="D9" s="7">
         <f>SUMIFS('Entrada e Saída'!E:E,'Entrada e Saída'!D:D,Saldo!$D$3,'Entrada e Saída'!C:C,Saldo!$B9)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E9" s="7">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" s="7" t="str">
         <f t="shared" si="1"/>
-        <v>Ok</v>
+        <v>Comprar</v>
       </c>
       <c r="H9" s="7"/>
     </row>
@@ -1118,15 +1164,15 @@
       </c>
       <c r="D13" s="7">
         <f>SUMIFS('Entrada e Saída'!E:E,'Entrada e Saída'!D:D,Saldo!$D$3,'Entrada e Saída'!C:C,Saldo!$B13)</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="F13" s="7" t="str">
         <f t="shared" si="1"/>
-        <v>Ok</v>
+        <v>Comprar</v>
       </c>
       <c r="H13" s="7"/>
     </row>
@@ -1241,6 +1287,11 @@
       <c r="H18" s="7"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B4:F18">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$F4="Comprar"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
desabilitando exibição de guias
Foi desabilitado a exibição das guias das planilhas Entrada e Saída, Menu e Saldo. No caminho opções do Excel -> avançado -> opções e exibição desta pasta de trabalho -> mostrar guias de planilha _> desabilitado.
</commit_message>
<xml_diff>
--- a/planilha de controle de estoque.xlsx
+++ b/planilha de controle de estoque.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Odirlei Guilherme\Desktop\controle_de_estoque_basico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD26C3DD-4E75-48E9-BC7E-91689E48033A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF1F3D1B-44F3-47A3-AAC2-07BF272311C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20280" yWindow="-135" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{FB90DC12-CE7E-421E-A7F9-F06FD8601840}"/>
+    <workbookView showSheetTabs="0" xWindow="20280" yWindow="-135" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{FB90DC12-CE7E-421E-A7F9-F06FD8601840}"/>
   </bookViews>
   <sheets>
     <sheet name="Entrada e Saída" sheetId="1" r:id="rId1"/>

</xml_diff>